<commit_message>
Add wishlist integration tests and update RTM with Sprint 4 requirements - close #123
</commit_message>
<xml_diff>
--- a/RTM_Switchr.xlsx
+++ b/RTM_Switchr.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,8 +33,12 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -61,8 +65,18 @@
         <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001a1a1a"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7F6F3"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -70,11 +84,17 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -92,6 +112,13 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -459,21 +486,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F156"/>
+  <dimension ref="A1:F167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Switchr - Requirements Traceability Matrix - CSE 4214 Sprint 3</t>
+          <t>Switchr - Requirements Traceability Matrix - CSE 4214 Sprint 4</t>
         </is>
       </c>
     </row>
@@ -5432,6 +5459,302 @@
         </is>
       </c>
       <c r="F156" s="6" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="157"/>
+    <row r="158">
+      <c r="A158" s="7" t="inlineStr">
+        <is>
+          <t>--- SPRINT 4 REQUIREMENTS ---</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="8" t="inlineStr">
+        <is>
+          <t>REQ-161</t>
+        </is>
+      </c>
+      <c r="B159" s="8" t="inlineStr">
+        <is>
+          <t>The system shall allow buyers to save listings to a personal wishlist.</t>
+        </is>
+      </c>
+      <c r="C159" s="8" t="inlineStr">
+        <is>
+          <t>US-17</t>
+        </is>
+      </c>
+      <c r="D159" s="8" t="inlineStr">
+        <is>
+          <t>#115</t>
+        </is>
+      </c>
+      <c r="E159" s="8" t="inlineStr">
+        <is>
+          <t>Integration_Testing/test_wishlist.py</t>
+        </is>
+      </c>
+      <c r="F159" s="8" t="inlineStr">
+        <is>
+          <t>11/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="9" t="inlineStr">
+        <is>
+          <t>REQ-162</t>
+        </is>
+      </c>
+      <c r="B160" s="9" t="inlineStr">
+        <is>
+          <t>The system shall allow buyers to view all saved wishlist items.</t>
+        </is>
+      </c>
+      <c r="C160" s="9" t="inlineStr">
+        <is>
+          <t>US-17</t>
+        </is>
+      </c>
+      <c r="D160" s="9" t="inlineStr">
+        <is>
+          <t>#115</t>
+        </is>
+      </c>
+      <c r="E160" s="9" t="inlineStr">
+        <is>
+          <t>Integration_Testing/test_wishlist.py</t>
+        </is>
+      </c>
+      <c r="F160" s="9" t="inlineStr">
+        <is>
+          <t>11/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="8" t="inlineStr">
+        <is>
+          <t>REQ-163</t>
+        </is>
+      </c>
+      <c r="B161" s="8" t="inlineStr">
+        <is>
+          <t>The system shall allow buyers to remove items from their wishlist.</t>
+        </is>
+      </c>
+      <c r="C161" s="8" t="inlineStr">
+        <is>
+          <t>US-17</t>
+        </is>
+      </c>
+      <c r="D161" s="8" t="inlineStr">
+        <is>
+          <t>#115</t>
+        </is>
+      </c>
+      <c r="E161" s="8" t="inlineStr">
+        <is>
+          <t>Integration_Testing/test_wishlist.py</t>
+        </is>
+      </c>
+      <c r="F161" s="8" t="inlineStr">
+        <is>
+          <t>11/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="9" t="inlineStr">
+        <is>
+          <t>REQ-164</t>
+        </is>
+      </c>
+      <c r="B162" s="9" t="inlineStr">
+        <is>
+          <t>The system shall prevent duplicate entries in a buyers wishlist.</t>
+        </is>
+      </c>
+      <c r="C162" s="9" t="inlineStr">
+        <is>
+          <t>US-17</t>
+        </is>
+      </c>
+      <c r="D162" s="9" t="inlineStr">
+        <is>
+          <t>#115</t>
+        </is>
+      </c>
+      <c r="E162" s="9" t="inlineStr">
+        <is>
+          <t>Integration_Testing/test_wishlist.py</t>
+        </is>
+      </c>
+      <c r="F162" s="9" t="inlineStr">
+        <is>
+          <t>11/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="8" t="inlineStr">
+        <is>
+          <t>REQ-165</t>
+        </is>
+      </c>
+      <c r="B163" s="8" t="inlineStr">
+        <is>
+          <t>The system shall allow buyers to move wishlist items directly to cart.</t>
+        </is>
+      </c>
+      <c r="C163" s="8" t="inlineStr">
+        <is>
+          <t>US-17</t>
+        </is>
+      </c>
+      <c r="D163" s="8" t="inlineStr">
+        <is>
+          <t>#115</t>
+        </is>
+      </c>
+      <c r="E163" s="8" t="inlineStr">
+        <is>
+          <t>Integration_Testing/test_wishlist.py</t>
+        </is>
+      </c>
+      <c r="F163" s="8" t="inlineStr">
+        <is>
+          <t>11/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="9" t="inlineStr">
+        <is>
+          <t>REQ-166</t>
+        </is>
+      </c>
+      <c r="B164" s="9" t="inlineStr">
+        <is>
+          <t>The system shall automatically refresh seller notifications every 30 seconds without requiring a page reload.</t>
+        </is>
+      </c>
+      <c r="C164" s="9" t="inlineStr">
+        <is>
+          <t>US-18</t>
+        </is>
+      </c>
+      <c r="D164" s="9" t="inlineStr">
+        <is>
+          <t>#118</t>
+        </is>
+      </c>
+      <c r="E164" s="9" t="inlineStr">
+        <is>
+          <t>Integration_Testing/test_wishlist.py</t>
+        </is>
+      </c>
+      <c r="F164" s="9" t="inlineStr">
+        <is>
+          <t>11/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="8" t="inlineStr">
+        <is>
+          <t>REQ-167</t>
+        </is>
+      </c>
+      <c r="B165" s="8" t="inlineStr">
+        <is>
+          <t>The system shall block rendering of admin pages before authentication is verified to prevent race condition exposure.</t>
+        </is>
+      </c>
+      <c r="C165" s="8" t="inlineStr">
+        <is>
+          <t>US-14</t>
+        </is>
+      </c>
+      <c r="D165" s="8" t="inlineStr">
+        <is>
+          <t>#122</t>
+        </is>
+      </c>
+      <c r="E165" s="8" t="inlineStr">
+        <is>
+          <t>Integration_Testing/test_admin.py</t>
+        </is>
+      </c>
+      <c r="F165" s="8" t="inlineStr">
+        <is>
+          <t>13/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="9" t="inlineStr">
+        <is>
+          <t>REQ-168</t>
+        </is>
+      </c>
+      <c r="B166" s="9" t="inlineStr">
+        <is>
+          <t>The system shall apply a consistent UI color scheme and styling across all user roles including buyer, seller, and admin pages.</t>
+        </is>
+      </c>
+      <c r="C166" s="9" t="inlineStr">
+        <is>
+          <t>US-19</t>
+        </is>
+      </c>
+      <c r="D166" s="9" t="inlineStr">
+        <is>
+          <t>#120</t>
+        </is>
+      </c>
+      <c r="E166" s="9" t="inlineStr">
+        <is>
+          <t>N/A - UI Requirement</t>
+        </is>
+      </c>
+      <c r="F166" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="8" t="inlineStr">
+        <is>
+          <t>REQ-169</t>
+        </is>
+      </c>
+      <c r="B167" s="8" t="inlineStr">
+        <is>
+          <t>The system shall use shared CSS components for navigation, cards, typography, and status badges across all pages.</t>
+        </is>
+      </c>
+      <c r="C167" s="8" t="inlineStr">
+        <is>
+          <t>US-19</t>
+        </is>
+      </c>
+      <c r="D167" s="8" t="inlineStr">
+        <is>
+          <t>#121</t>
+        </is>
+      </c>
+      <c r="E167" s="8" t="inlineStr">
+        <is>
+          <t>N/A - UI Requirement</t>
+        </is>
+      </c>
+      <c r="F167" s="8" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>

</xml_diff>

<commit_message>
Update RTM with security testing requirements REQ-170 to REQ-176 - ref #127
</commit_message>
<xml_diff>
--- a/RTM_Switchr.xlsx
+++ b/RTM_Switchr.xlsx
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F167"/>
+  <dimension ref="A1:F174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5464,7 +5464,6 @@
         </is>
       </c>
     </row>
-    <row r="157"/>
     <row r="158">
       <c r="A158" s="7" t="inlineStr">
         <is>
@@ -5757,6 +5756,230 @@
       <c r="F167" s="8" t="inlineStr">
         <is>
           <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="8" t="inlineStr">
+        <is>
+          <t>REQ-170</t>
+        </is>
+      </c>
+      <c r="B168" s="8" t="inlineStr">
+        <is>
+          <t>The system shall reject SQL injection attempts in the login email and password fields.</t>
+        </is>
+      </c>
+      <c r="C168" s="8" t="inlineStr">
+        <is>
+          <t>US-22</t>
+        </is>
+      </c>
+      <c r="D168" s="8" t="inlineStr">
+        <is>
+          <t>#127</t>
+        </is>
+      </c>
+      <c r="E168" s="8" t="inlineStr">
+        <is>
+          <t>Integration_Testing/test_security.py</t>
+        </is>
+      </c>
+      <c r="F168" s="8" t="inlineStr">
+        <is>
+          <t>19/19</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="9" t="inlineStr">
+        <is>
+          <t>REQ-171</t>
+        </is>
+      </c>
+      <c r="B169" s="9" t="inlineStr">
+        <is>
+          <t>The system shall reject SQL injection attempts in the search and listing ID parameters.</t>
+        </is>
+      </c>
+      <c r="C169" s="9" t="inlineStr">
+        <is>
+          <t>US-22</t>
+        </is>
+      </c>
+      <c r="D169" s="9" t="inlineStr">
+        <is>
+          <t>#127</t>
+        </is>
+      </c>
+      <c r="E169" s="9" t="inlineStr">
+        <is>
+          <t>Integration_Testing/test_security.py</t>
+        </is>
+      </c>
+      <c r="F169" s="9" t="inlineStr">
+        <is>
+          <t>19/19</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="8" t="inlineStr">
+        <is>
+          <t>REQ-172</t>
+        </is>
+      </c>
+      <c r="B170" s="8" t="inlineStr">
+        <is>
+          <t>The system shall reject all requests to protected routes that do not include a valid authentication token.</t>
+        </is>
+      </c>
+      <c r="C170" s="8" t="inlineStr">
+        <is>
+          <t>US-22</t>
+        </is>
+      </c>
+      <c r="D170" s="8" t="inlineStr">
+        <is>
+          <t>#127</t>
+        </is>
+      </c>
+      <c r="E170" s="8" t="inlineStr">
+        <is>
+          <t>Integration_Testing/test_security.py</t>
+        </is>
+      </c>
+      <c r="F170" s="8" t="inlineStr">
+        <is>
+          <t>19/19</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="9" t="inlineStr">
+        <is>
+          <t>REQ-173</t>
+        </is>
+      </c>
+      <c r="B171" s="9" t="inlineStr">
+        <is>
+          <t>The system shall reject malformed or invalid authorization headers with a 401 response.</t>
+        </is>
+      </c>
+      <c r="C171" s="9" t="inlineStr">
+        <is>
+          <t>US-22</t>
+        </is>
+      </c>
+      <c r="D171" s="9" t="inlineStr">
+        <is>
+          <t>#127</t>
+        </is>
+      </c>
+      <c r="E171" s="9" t="inlineStr">
+        <is>
+          <t>Integration_Testing/test_security.py</t>
+        </is>
+      </c>
+      <c r="F171" s="9" t="inlineStr">
+        <is>
+          <t>19/19</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="8" t="inlineStr">
+        <is>
+          <t>REQ-174</t>
+        </is>
+      </c>
+      <c r="B172" s="8" t="inlineStr">
+        <is>
+          <t>The system shall prevent non-admin users from accessing admin endpoints.</t>
+        </is>
+      </c>
+      <c r="C172" s="8" t="inlineStr">
+        <is>
+          <t>US-22</t>
+        </is>
+      </c>
+      <c r="D172" s="8" t="inlineStr">
+        <is>
+          <t>#127</t>
+        </is>
+      </c>
+      <c r="E172" s="8" t="inlineStr">
+        <is>
+          <t>Integration_Testing/test_security.py</t>
+        </is>
+      </c>
+      <c r="F172" s="8" t="inlineStr">
+        <is>
+          <t>19/19</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="9" t="inlineStr">
+        <is>
+          <t>REQ-175</t>
+        </is>
+      </c>
+      <c r="B173" s="9" t="inlineStr">
+        <is>
+          <t>The system shall prevent sellers from editing listings they do not own.</t>
+        </is>
+      </c>
+      <c r="C173" s="9" t="inlineStr">
+        <is>
+          <t>US-22</t>
+        </is>
+      </c>
+      <c r="D173" s="9" t="inlineStr">
+        <is>
+          <t>#127</t>
+        </is>
+      </c>
+      <c r="E173" s="9" t="inlineStr">
+        <is>
+          <t>Integration_Testing/test_security.py</t>
+        </is>
+      </c>
+      <c r="F173" s="9" t="inlineStr">
+        <is>
+          <t>19/19</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="8" t="inlineStr">
+        <is>
+          <t>REQ-176</t>
+        </is>
+      </c>
+      <c r="B174" s="8" t="inlineStr">
+        <is>
+          <t>The system shall handle XSS payloads in user input fields without crashing or exposing data.</t>
+        </is>
+      </c>
+      <c r="C174" s="8" t="inlineStr">
+        <is>
+          <t>US-22</t>
+        </is>
+      </c>
+      <c r="D174" s="8" t="inlineStr">
+        <is>
+          <t>#127</t>
+        </is>
+      </c>
+      <c r="E174" s="8" t="inlineStr">
+        <is>
+          <t>Integration_Testing/test_security.py</t>
+        </is>
+      </c>
+      <c r="F174" s="8" t="inlineStr">
+        <is>
+          <t>19/19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update RTM with auction requirements REQ-177 to REQ-182 - ref #135
</commit_message>
<xml_diff>
--- a/RTM_Switchr.xlsx
+++ b/RTM_Switchr.xlsx
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F174"/>
+  <dimension ref="A1:F180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5983,6 +5983,198 @@
         </is>
       </c>
     </row>
+    <row r="175">
+      <c r="A175" s="8" t="inlineStr">
+        <is>
+          <t>REQ-177</t>
+        </is>
+      </c>
+      <c r="B175" s="8" t="inlineStr">
+        <is>
+          <t>The system shall allow sellers to create auction listings with a starting price and duration of 1, 3, or 7 days.</t>
+        </is>
+      </c>
+      <c r="C175" s="8" t="inlineStr">
+        <is>
+          <t>US-22</t>
+        </is>
+      </c>
+      <c r="D175" s="8" t="inlineStr">
+        <is>
+          <t>#117</t>
+        </is>
+      </c>
+      <c r="E175" s="8" t="inlineStr">
+        <is>
+          <t>Integration_Testing/test_auction.py</t>
+        </is>
+      </c>
+      <c r="F175" s="8" t="inlineStr">
+        <is>
+          <t>12/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="9" t="inlineStr">
+        <is>
+          <t>REQ-178</t>
+        </is>
+      </c>
+      <c r="B176" s="9" t="inlineStr">
+        <is>
+          <t>The system shall allow approved buyers to place bids on active auction listings.</t>
+        </is>
+      </c>
+      <c r="C176" s="9" t="inlineStr">
+        <is>
+          <t>US-22</t>
+        </is>
+      </c>
+      <c r="D176" s="9" t="inlineStr">
+        <is>
+          <t>#117</t>
+        </is>
+      </c>
+      <c r="E176" s="9" t="inlineStr">
+        <is>
+          <t>Integration_Testing/test_auction.py</t>
+        </is>
+      </c>
+      <c r="F176" s="9" t="inlineStr">
+        <is>
+          <t>12/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="8" t="inlineStr">
+        <is>
+          <t>REQ-179</t>
+        </is>
+      </c>
+      <c r="B177" s="8" t="inlineStr">
+        <is>
+          <t>The system shall reject bids that do not exceed the current highest bid price.</t>
+        </is>
+      </c>
+      <c r="C177" s="8" t="inlineStr">
+        <is>
+          <t>US-22</t>
+        </is>
+      </c>
+      <c r="D177" s="8" t="inlineStr">
+        <is>
+          <t>#117</t>
+        </is>
+      </c>
+      <c r="E177" s="8" t="inlineStr">
+        <is>
+          <t>Integration_Testing/test_auction.py</t>
+        </is>
+      </c>
+      <c r="F177" s="8" t="inlineStr">
+        <is>
+          <t>12/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="9" t="inlineStr">
+        <is>
+          <t>REQ-180</t>
+        </is>
+      </c>
+      <c r="B178" s="9" t="inlineStr">
+        <is>
+          <t>The system shall prevent sellers from placing bids on their own auction listings.</t>
+        </is>
+      </c>
+      <c r="C178" s="9" t="inlineStr">
+        <is>
+          <t>US-22</t>
+        </is>
+      </c>
+      <c r="D178" s="9" t="inlineStr">
+        <is>
+          <t>#117</t>
+        </is>
+      </c>
+      <c r="E178" s="9" t="inlineStr">
+        <is>
+          <t>Integration_Testing/test_auction.py</t>
+        </is>
+      </c>
+      <c r="F178" s="9" t="inlineStr">
+        <is>
+          <t>12/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" s="8" t="inlineStr">
+        <is>
+          <t>REQ-181</t>
+        </is>
+      </c>
+      <c r="B179" s="8" t="inlineStr">
+        <is>
+          <t>The system shall notify the previous highest bidder when they are outbid.</t>
+        </is>
+      </c>
+      <c r="C179" s="8" t="inlineStr">
+        <is>
+          <t>US-22</t>
+        </is>
+      </c>
+      <c r="D179" s="8" t="inlineStr">
+        <is>
+          <t>#117</t>
+        </is>
+      </c>
+      <c r="E179" s="8" t="inlineStr">
+        <is>
+          <t>Integration_Testing/test_auction.py</t>
+        </is>
+      </c>
+      <c r="F179" s="8" t="inlineStr">
+        <is>
+          <t>12/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="9" t="inlineStr">
+        <is>
+          <t>REQ-182</t>
+        </is>
+      </c>
+      <c r="B180" s="9" t="inlineStr">
+        <is>
+          <t>The system shall settle expired auctions lazily when they are next viewed or bid on.</t>
+        </is>
+      </c>
+      <c r="C180" s="9" t="inlineStr">
+        <is>
+          <t>US-22</t>
+        </is>
+      </c>
+      <c r="D180" s="9" t="inlineStr">
+        <is>
+          <t>#117</t>
+        </is>
+      </c>
+      <c r="E180" s="9" t="inlineStr">
+        <is>
+          <t>Integration_Testing/test_auction.py</t>
+        </is>
+      </c>
+      <c r="F180" s="9" t="inlineStr">
+        <is>
+          <t>12/12</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>